<commit_message>
exp max new tokens reg test v2
</commit_message>
<xml_diff>
--- a/results/reliability_eval/reliability_eval_09-17-1-regenerated-v2/scores_Llama-3-8B_P101_0_sample_45_tokens_0.1_temp_direct_completion_raw_table_09-17-1.xlsx_updated.xlsx
+++ b/results/reliability_eval/reliability_eval_09-17-1-regenerated-v2/scores_Llama-3-8B_P101_0_sample_45_tokens_0.1_temp_direct_completion_raw_table_09-17-1.xlsx_updated.xlsx
@@ -425,138 +425,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>AUCROC_sample</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>AUCPR_sample</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Brier_sample</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>LogLoss_sample</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Entropy_sample</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>AUCROC_adj</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>AUCPR_adj</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Brier_adj</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>LogLoss_adj</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Entropy_adj</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>AUCROC_sem</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>AUCPR_sem</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Brier_sem</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>LogLoss_sem</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Entropy_sem</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Accuracy</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
         <v>0.7792305383718793</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>0.7188673884510498</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>0.2056062947342136</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>2.795385774978577</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>1938.382755650759</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0.6373199425291749</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.6565441931528483</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>0.509316716045793</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>4.053507124394018</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>334.6009896463219</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.9883831959987117</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>0.9845927476871189</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>0.0435919540229885</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>0.1301247070989476</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>659.8223917058774</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>0.460632183908046</v>
       </c>
     </row>

</xml_diff>